<commit_message>
Add flag_multi_rn_dinas + Hornschuch Accuracy_PRE sheet
- net_dinas_fracht(): new flag_multi_rn_dinas = (n_rows_per_snr > 1)
  detects re-invoicing artifacts where netto_total is inflated (2x/3x)
- enrich_customer_bi(): exclude multi-row SNRs from ±5% accuracy base;
  adds n_multi_rn_dinas, n_acc_base to stats dict
- build_cht_report: DQ block shows D) DINAS Multi-Row exclusion;
  Accuracy_PRE marks multi-row rows in orange; column N=37
- build_hornschuch_report: full BI enrichment integration (Komplettpreis,
  Sammelposten, Gutschrift-Netting, Multi-Row flag); new DQ block on
  Sheet 1; new Sheet 3 Accuracy_PRE (1365 rows, 926/940 = 98.5% ±5%)
  CHT: 91/93 = 97.8% clean base after 5 multi-row exclusions
  Hornschuch: 425/1365 multi-row flagged, 926/940 = 98.5% clean base

https://claude.ai/code/session_01QY1f1VNnd5RWsUcy3L3Squ
</commit_message>
<xml_diff>
--- a/output/billing_report/cht_dinas_vergleich.xlsx
+++ b/output/billing_report/cht_dinas_vergleich.xlsx
@@ -61,7 +61,7 @@
       <sz val="10"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +105,11 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00FFCC99"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
@@ -135,7 +140,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -204,6 +209,18 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="3" fillId="10" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="164" fontId="3" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -577,7 +594,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AJ45"/>
+  <dimension ref="A1:AK45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -616,6 +633,7 @@
     <col width="10" customWidth="1" min="34" max="34"/>
     <col width="8" customWidth="1" min="35" max="35"/>
     <col width="10" customWidth="1" min="36" max="36"/>
+    <col width="12" customWidth="1" min="37" max="37"/>
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
@@ -659,12 +677,12 @@
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
         <is>
-          <t>davon im ±5%-Band</t>
+          <t>davon im ±5%-Band (ex. DINAS Multi-Row)</t>
         </is>
       </c>
       <c r="S5" s="4" t="inlineStr">
         <is>
-          <t>96 / 98 (98%)  ← Basis-Accuracy</t>
+          <t>91 / 92 (99% der Acc.-Basis)  ← Basis-Accuracy</t>
         </is>
       </c>
     </row>
@@ -676,7 +694,7 @@
       </c>
       <c r="S6" s="4" t="inlineStr">
         <is>
-          <t>A) Komplettpreis ohne DINAS-Match: 619 SNRs  |  B) Sammelposten (strukturell, nicht ausgeschlossen): 1414 SNRs (94%)  |  C) Solo-Gutschriften: 8</t>
+          <t>A) Kein DINAS-Match: 619 SNRs  |  B) Sammelposten (strukturell, nicht ausgeschlossen): 1414 SNRs (94%)  |  C) Solo-Gutschriften: 8  |  D) DINAS Multi-Row: 6 SNRs (aus ±5%-Basis ausgeschlossen)</t>
         </is>
       </c>
     </row>
@@ -871,6 +889,11 @@
       <c r="AJ8" s="5" t="inlineStr">
         <is>
           <t>DINAS vs BI %</t>
+        </is>
+      </c>
+      <c r="AK8" s="5" t="inlineStr">
+        <is>
+          <t>DINAS Multi-Row</t>
         </is>
       </c>
     </row>
@@ -1002,6 +1025,7 @@
       <c r="AJ10" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="AK10" s="7" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
@@ -1118,6 +1142,7 @@
       <c r="AH11" s="11" t="inlineStr"/>
       <c r="AI11" s="11" t="inlineStr"/>
       <c r="AJ11" s="12" t="n"/>
+      <c r="AK11" s="11" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
@@ -1238,6 +1263,7 @@
         </is>
       </c>
       <c r="AJ12" s="8" t="n"/>
+      <c r="AK12" s="7" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
@@ -1363,6 +1389,7 @@
       <c r="AJ15" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="AK15" s="15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
@@ -1485,6 +1512,7 @@
       <c r="AJ16" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="AK16" s="15" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
@@ -1607,6 +1635,11 @@
       <c r="AJ17" s="16" t="n">
         <v>1483.08</v>
       </c>
+      <c r="AK17" s="15" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
@@ -1729,6 +1762,11 @@
       <c r="AJ18" s="16" t="n">
         <v>1483.08</v>
       </c>
+      <c r="AK18" s="15" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
@@ -1851,6 +1889,7 @@
       <c r="AJ19" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="AK19" s="15" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
@@ -1971,6 +2010,7 @@
         </is>
       </c>
       <c r="AJ20" s="8" t="n"/>
+      <c r="AK20" s="7" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="inlineStr">
@@ -2100,6 +2140,7 @@
       <c r="AJ23" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="AK23" s="7" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="11" t="inlineStr">
@@ -2220,6 +2261,7 @@
         </is>
       </c>
       <c r="AJ24" s="12" t="n"/>
+      <c r="AK24" s="11" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="11" t="inlineStr">
@@ -2340,6 +2382,7 @@
         </is>
       </c>
       <c r="AJ25" s="12" t="n"/>
+      <c r="AK25" s="11" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="11" t="inlineStr">
@@ -2460,6 +2503,7 @@
         </is>
       </c>
       <c r="AJ26" s="12" t="n"/>
+      <c r="AK26" s="11" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="7" t="inlineStr">
@@ -2580,6 +2624,7 @@
         </is>
       </c>
       <c r="AJ27" s="8" t="n"/>
+      <c r="AK27" s="7" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="11" t="inlineStr">
@@ -2700,6 +2745,7 @@
         </is>
       </c>
       <c r="AJ28" s="12" t="n"/>
+      <c r="AK28" s="11" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="inlineStr">
@@ -2825,6 +2871,7 @@
       <c r="AJ31" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="AK31" s="7" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
@@ -2947,6 +2994,7 @@
       <c r="AJ32" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="AK32" s="15" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="15" t="inlineStr">
@@ -3069,6 +3117,7 @@
       <c r="AJ33" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="AK33" s="15" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="15" t="inlineStr">
@@ -3191,6 +3240,7 @@
       <c r="AJ34" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="AK34" s="15" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="15" t="inlineStr">
@@ -3313,6 +3363,7 @@
       <c r="AJ35" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="AK35" s="15" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="7" t="inlineStr">
@@ -3433,6 +3484,7 @@
         </is>
       </c>
       <c r="AJ36" s="8" t="n"/>
+      <c r="AK36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
@@ -3553,6 +3605,7 @@
         </is>
       </c>
       <c r="AJ37" s="12" t="n"/>
+      <c r="AK37" s="11" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="11" t="inlineStr">
@@ -3673,6 +3726,7 @@
         </is>
       </c>
       <c r="AJ38" s="12" t="n"/>
+      <c r="AK38" s="11" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="11" t="inlineStr">
@@ -3793,6 +3847,7 @@
         </is>
       </c>
       <c r="AJ39" s="12" t="n"/>
+      <c r="AK39" s="11" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="11" t="inlineStr">
@@ -3913,6 +3968,7 @@
         </is>
       </c>
       <c r="AJ40" s="12" t="n"/>
+      <c r="AK40" s="11" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
@@ -4042,6 +4098,7 @@
       <c r="AJ43" s="8" t="n">
         <v>0</v>
       </c>
+      <c r="AK43" s="7" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="15" t="inlineStr">
@@ -4164,6 +4221,7 @@
       <c r="AJ44" s="16" t="n">
         <v>0</v>
       </c>
+      <c r="AK44" s="15" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="7" t="inlineStr">
@@ -4284,25 +4342,26 @@
         </is>
       </c>
       <c r="AJ45" s="8" t="n"/>
+      <c r="AK45" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="17">
     <mergeCell ref="A3:R3"/>
-    <mergeCell ref="A1:AJ1"/>
-    <mergeCell ref="A14:AJ14"/>
+    <mergeCell ref="S7:AK7"/>
+    <mergeCell ref="S5:AK5"/>
+    <mergeCell ref="A30:AK30"/>
     <mergeCell ref="A7:R7"/>
-    <mergeCell ref="A22:AJ22"/>
-    <mergeCell ref="A9:AJ9"/>
-    <mergeCell ref="S7:AJ7"/>
+    <mergeCell ref="S6:AK6"/>
+    <mergeCell ref="A22:AK22"/>
     <mergeCell ref="A2:R2"/>
-    <mergeCell ref="S5:AJ5"/>
-    <mergeCell ref="A30:AJ30"/>
-    <mergeCell ref="S6:AJ6"/>
+    <mergeCell ref="S4:AK4"/>
+    <mergeCell ref="A42:AK42"/>
+    <mergeCell ref="S3:AK3"/>
+    <mergeCell ref="A5:R5"/>
+    <mergeCell ref="A14:AK14"/>
+    <mergeCell ref="A1:AK1"/>
+    <mergeCell ref="A9:AK9"/>
     <mergeCell ref="A6:R6"/>
-    <mergeCell ref="A5:R5"/>
-    <mergeCell ref="A42:AJ42"/>
-    <mergeCell ref="S3:AJ3"/>
-    <mergeCell ref="S4:AJ4"/>
     <mergeCell ref="A4:R4"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5427,7 +5486,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O100"/>
+  <dimension ref="A1:P100"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -5444,13 +5503,14 @@
     <col width="10" customWidth="1" min="12" max="12"/>
     <col width="8" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
   </cols>
   <sheetData>
     <row r="1" ht="18" customHeight="1">
       <c r="A1" s="19" t="inlineStr">
         <is>
-          <t>CHT Germany GmbH (486073) — PRE Accuracy: DINAS Total (Komplettpreis-Fix) vs BI Erloese_effektiv  |  Rows: 98  |  ±5%: 96 (98%)  |  &gt;10% Abw.: 2  |  Komplettpreis: 98  |  Sammelposten: 90  |  Solo-Gutschrift: 0  |  [Alt ohne Komplettpreis-Fix: 0 vergleichbar]</t>
+          <t>CHT Germany GmbH (486073) — PRE Accuracy: DINAS Total (Komplettpreis-Fix) vs BI Erloese_effektiv  |  Rows: 98  |  Multi-Row (ausgeschl.): 6  |  Acc.-Basis: 92  |  ±5%: 91 (99% der Basis)  |  &gt;10% Abw.: 1  |  Komplettpreis: 98  |  Sammelposten: 90  |  Solo-Gutschrift: 0</t>
         </is>
       </c>
     </row>
@@ -5527,6 +5587,11 @@
       </c>
       <c r="O2" s="5" t="inlineStr">
         <is>
+          <t>Multi-Row DINAS</t>
+        </is>
+      </c>
+      <c r="P2" s="5" t="inlineStr">
+        <is>
           <t>Abw. Klasse</t>
         </is>
       </c>
@@ -5588,66 +5653,72 @@
       <c r="N3" s="20" t="inlineStr"/>
       <c r="O3" s="20" t="inlineStr">
         <is>
-          <t>&gt;10%</t>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="P3" s="20" t="inlineStr">
+        <is>
+          <t>Multi-Row</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="24" t="inlineStr">
         <is>
           <t>32904834</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="24" t="inlineStr">
         <is>
           <t>3767265</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="24" t="inlineStr">
         <is>
           <t>53013296</t>
         </is>
       </c>
-      <c r="D4" s="21" t="n">
+      <c r="D4" s="25" t="n">
         <v>45811</v>
       </c>
-      <c r="E4" s="20" t="inlineStr">
+      <c r="E4" s="24" t="inlineStr">
         <is>
           <t>IT</t>
         </is>
       </c>
-      <c r="F4" s="20" t="inlineStr">
+      <c r="F4" s="24" t="inlineStr">
         <is>
           <t xml:space="preserve">24050    </t>
         </is>
       </c>
-      <c r="G4" s="20" t="n">
+      <c r="G4" s="24" t="n">
         <v>9576</v>
       </c>
-      <c r="H4" s="22" t="n">
+      <c r="H4" s="26" t="n">
         <v>100</v>
       </c>
-      <c r="I4" s="22" t="n">
+      <c r="I4" s="26" t="n">
         <v>944.6</v>
       </c>
-      <c r="J4" s="22" t="n">
+      <c r="J4" s="26" t="n">
         <v>-844.6</v>
       </c>
-      <c r="K4" s="23" t="n">
+      <c r="K4" s="27" t="n">
         <v>-89.40000000000001</v>
       </c>
-      <c r="L4" s="20" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="M4" s="20" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="N4" s="20" t="inlineStr"/>
-      <c r="O4" s="20" t="inlineStr">
+      <c r="L4" s="24" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M4" s="24" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="N4" s="24" t="inlineStr"/>
+      <c r="O4" s="24" t="inlineStr"/>
+      <c r="P4" s="24" t="inlineStr">
         <is>
           <t>&gt;10%</t>
         </is>
@@ -5669,7 +5740,7 @@
           <t>53013248</t>
         </is>
       </c>
-      <c r="D5" s="24" t="n">
+      <c r="D5" s="28" t="n">
         <v>45776</v>
       </c>
       <c r="E5" s="7" t="inlineStr">
@@ -5694,7 +5765,7 @@
       <c r="J5" s="10" t="n">
         <v>-0.99</v>
       </c>
-      <c r="K5" s="25" t="n">
+      <c r="K5" s="29" t="n">
         <v>-0.7</v>
       </c>
       <c r="L5" s="7" t="inlineStr">
@@ -5708,7 +5779,8 @@
         </is>
       </c>
       <c r="N5" s="7" t="inlineStr"/>
-      <c r="O5" s="7" t="inlineStr">
+      <c r="O5" s="7" t="inlineStr"/>
+      <c r="P5" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -5730,7 +5802,7 @@
           <t>53013248</t>
         </is>
       </c>
-      <c r="D6" s="24" t="n">
+      <c r="D6" s="28" t="n">
         <v>45776</v>
       </c>
       <c r="E6" s="7" t="inlineStr">
@@ -5755,7 +5827,7 @@
       <c r="J6" s="10" t="n">
         <v>-1.87</v>
       </c>
-      <c r="K6" s="25" t="n">
+      <c r="K6" s="29" t="n">
         <v>-0.7</v>
       </c>
       <c r="L6" s="7" t="inlineStr">
@@ -5769,7 +5841,8 @@
         </is>
       </c>
       <c r="N6" s="7" t="inlineStr"/>
-      <c r="O6" s="7" t="inlineStr">
+      <c r="O6" s="7" t="inlineStr"/>
+      <c r="P6" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -5791,7 +5864,7 @@
           <t>53013250</t>
         </is>
       </c>
-      <c r="D7" s="24" t="n">
+      <c r="D7" s="28" t="n">
         <v>45775</v>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -5816,7 +5889,7 @@
       <c r="J7" s="10" t="n">
         <v>-1.47</v>
       </c>
-      <c r="K7" s="25" t="n">
+      <c r="K7" s="29" t="n">
         <v>-0.5</v>
       </c>
       <c r="L7" s="7" t="inlineStr">
@@ -5830,7 +5903,8 @@
         </is>
       </c>
       <c r="N7" s="7" t="inlineStr"/>
-      <c r="O7" s="7" t="inlineStr">
+      <c r="O7" s="7" t="inlineStr"/>
+      <c r="P7" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -5852,7 +5926,7 @@
           <t>53013250</t>
         </is>
       </c>
-      <c r="D8" s="24" t="n">
+      <c r="D8" s="28" t="n">
         <v>45775</v>
       </c>
       <c r="E8" s="7" t="inlineStr">
@@ -5877,7 +5951,7 @@
       <c r="J8" s="10" t="n">
         <v>-0.18</v>
       </c>
-      <c r="K8" s="25" t="n">
+      <c r="K8" s="29" t="n">
         <v>-0.5</v>
       </c>
       <c r="L8" s="7" t="inlineStr">
@@ -5891,7 +5965,8 @@
         </is>
       </c>
       <c r="N8" s="7" t="inlineStr"/>
-      <c r="O8" s="7" t="inlineStr">
+      <c r="O8" s="7" t="inlineStr"/>
+      <c r="P8" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -5913,7 +5988,7 @@
           <t>53013250</t>
         </is>
       </c>
-      <c r="D9" s="24" t="n">
+      <c r="D9" s="28" t="n">
         <v>45775</v>
       </c>
       <c r="E9" s="7" t="inlineStr">
@@ -5938,7 +6013,7 @@
       <c r="J9" s="10" t="n">
         <v>-0.27</v>
       </c>
-      <c r="K9" s="25" t="n">
+      <c r="K9" s="29" t="n">
         <v>-0.5</v>
       </c>
       <c r="L9" s="7" t="inlineStr">
@@ -5952,7 +6027,8 @@
         </is>
       </c>
       <c r="N9" s="7" t="inlineStr"/>
-      <c r="O9" s="7" t="inlineStr">
+      <c r="O9" s="7" t="inlineStr"/>
+      <c r="P9" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -5974,7 +6050,7 @@
           <t>3759502</t>
         </is>
       </c>
-      <c r="D10" s="24" t="n">
+      <c r="D10" s="28" t="n">
         <v>45757</v>
       </c>
       <c r="E10" s="7" t="inlineStr">
@@ -5999,7 +6075,7 @@
       <c r="J10" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K10" s="25" t="n">
+      <c r="K10" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L10" s="7" t="inlineStr">
@@ -6009,70 +6085,76 @@
       </c>
       <c r="M10" s="7" t="inlineStr"/>
       <c r="N10" s="7" t="inlineStr"/>
-      <c r="O10" s="7" t="inlineStr">
+      <c r="O10" s="7" t="inlineStr"/>
+      <c r="P10" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>32877497</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>3759501</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>3759501</t>
         </is>
       </c>
-      <c r="D11" s="24" t="n">
+      <c r="D11" s="21" t="n">
         <v>45757</v>
       </c>
-      <c r="E11" s="7" t="inlineStr">
-        <is>
-          <t>GR</t>
-        </is>
-      </c>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="E11" s="20" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+      <c r="F11" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">57001    </t>
         </is>
       </c>
-      <c r="G11" s="7" t="n">
+      <c r="G11" s="20" t="n">
         <v>13594</v>
       </c>
-      <c r="H11" s="10" t="n">
+      <c r="H11" s="22" t="n">
         <v>3136.04</v>
       </c>
-      <c r="I11" s="10" t="n">
+      <c r="I11" s="22" t="n">
         <v>3136.04</v>
       </c>
-      <c r="J11" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K11" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="7" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="M11" s="7" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="N11" s="7" t="inlineStr"/>
-      <c r="O11" s="7" t="inlineStr">
-        <is>
-          <t>±5%</t>
+      <c r="J11" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K11" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M11" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="N11" s="20" t="inlineStr"/>
+      <c r="O11" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="P11" s="20" t="inlineStr">
+        <is>
+          <t>Multi-Row</t>
         </is>
       </c>
     </row>
@@ -6092,7 +6174,7 @@
           <t>3758675</t>
         </is>
       </c>
-      <c r="D12" s="24" t="n">
+      <c r="D12" s="28" t="n">
         <v>45750</v>
       </c>
       <c r="E12" s="7" t="inlineStr">
@@ -6117,7 +6199,7 @@
       <c r="J12" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K12" s="25" t="n">
+      <c r="K12" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L12" s="7" t="inlineStr">
@@ -6127,7 +6209,8 @@
       </c>
       <c r="M12" s="7" t="inlineStr"/>
       <c r="N12" s="7" t="inlineStr"/>
-      <c r="O12" s="7" t="inlineStr">
+      <c r="O12" s="7" t="inlineStr"/>
+      <c r="P12" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6149,7 +6232,7 @@
           <t>3760513</t>
         </is>
       </c>
-      <c r="D13" s="24" t="n">
+      <c r="D13" s="28" t="n">
         <v>45764</v>
       </c>
       <c r="E13" s="7" t="inlineStr">
@@ -6174,7 +6257,7 @@
       <c r="J13" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K13" s="25" t="n">
+      <c r="K13" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L13" s="7" t="inlineStr">
@@ -6188,7 +6271,8 @@
         </is>
       </c>
       <c r="N13" s="7" t="inlineStr"/>
-      <c r="O13" s="7" t="inlineStr">
+      <c r="O13" s="7" t="inlineStr"/>
+      <c r="P13" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6210,7 +6294,7 @@
           <t>3760513</t>
         </is>
       </c>
-      <c r="D14" s="24" t="n">
+      <c r="D14" s="28" t="n">
         <v>45764</v>
       </c>
       <c r="E14" s="7" t="inlineStr">
@@ -6235,7 +6319,7 @@
       <c r="J14" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K14" s="25" t="n">
+      <c r="K14" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="7" t="inlineStr">
@@ -6249,7 +6333,8 @@
         </is>
       </c>
       <c r="N14" s="7" t="inlineStr"/>
-      <c r="O14" s="7" t="inlineStr">
+      <c r="O14" s="7" t="inlineStr"/>
+      <c r="P14" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6271,7 +6356,7 @@
           <t>3760513</t>
         </is>
       </c>
-      <c r="D15" s="24" t="n">
+      <c r="D15" s="28" t="n">
         <v>45764</v>
       </c>
       <c r="E15" s="7" t="inlineStr">
@@ -6296,7 +6381,7 @@
       <c r="J15" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K15" s="25" t="n">
+      <c r="K15" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L15" s="7" t="inlineStr">
@@ -6310,7 +6395,8 @@
         </is>
       </c>
       <c r="N15" s="7" t="inlineStr"/>
-      <c r="O15" s="7" t="inlineStr">
+      <c r="O15" s="7" t="inlineStr"/>
+      <c r="P15" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6332,7 +6418,7 @@
           <t>3760512</t>
         </is>
       </c>
-      <c r="D16" s="24" t="n">
+      <c r="D16" s="28" t="n">
         <v>45763</v>
       </c>
       <c r="E16" s="7" t="inlineStr">
@@ -6357,7 +6443,7 @@
       <c r="J16" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K16" s="25" t="n">
+      <c r="K16" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="7" t="inlineStr">
@@ -6371,7 +6457,8 @@
         </is>
       </c>
       <c r="N16" s="7" t="inlineStr"/>
-      <c r="O16" s="7" t="inlineStr">
+      <c r="O16" s="7" t="inlineStr"/>
+      <c r="P16" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6393,7 +6480,7 @@
           <t>3760512</t>
         </is>
       </c>
-      <c r="D17" s="24" t="n">
+      <c r="D17" s="28" t="n">
         <v>45763</v>
       </c>
       <c r="E17" s="7" t="inlineStr">
@@ -6418,7 +6505,7 @@
       <c r="J17" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K17" s="25" t="n">
+      <c r="K17" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L17" s="7" t="inlineStr">
@@ -6432,7 +6519,8 @@
         </is>
       </c>
       <c r="N17" s="7" t="inlineStr"/>
-      <c r="O17" s="7" t="inlineStr">
+      <c r="O17" s="7" t="inlineStr"/>
+      <c r="P17" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6454,7 +6542,7 @@
           <t>3761610</t>
         </is>
       </c>
-      <c r="D18" s="24" t="n">
+      <c r="D18" s="28" t="n">
         <v>45772</v>
       </c>
       <c r="E18" s="7" t="inlineStr">
@@ -6479,7 +6567,7 @@
       <c r="J18" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K18" s="25" t="n">
+      <c r="K18" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="7" t="inlineStr">
@@ -6489,7 +6577,8 @@
       </c>
       <c r="M18" s="7" t="inlineStr"/>
       <c r="N18" s="7" t="inlineStr"/>
-      <c r="O18" s="7" t="inlineStr">
+      <c r="O18" s="7" t="inlineStr"/>
+      <c r="P18" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6511,7 +6600,7 @@
           <t>3760511</t>
         </is>
       </c>
-      <c r="D19" s="24" t="n">
+      <c r="D19" s="28" t="n">
         <v>45763</v>
       </c>
       <c r="E19" s="7" t="inlineStr">
@@ -6536,7 +6625,7 @@
       <c r="J19" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K19" s="25" t="n">
+      <c r="K19" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L19" s="7" t="inlineStr">
@@ -6546,7 +6635,8 @@
       </c>
       <c r="M19" s="7" t="inlineStr"/>
       <c r="N19" s="7" t="inlineStr"/>
-      <c r="O19" s="7" t="inlineStr">
+      <c r="O19" s="7" t="inlineStr"/>
+      <c r="P19" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6568,7 +6658,7 @@
           <t>3759501</t>
         </is>
       </c>
-      <c r="D20" s="24" t="n">
+      <c r="D20" s="28" t="n">
         <v>45757</v>
       </c>
       <c r="E20" s="7" t="inlineStr">
@@ -6593,7 +6683,7 @@
       <c r="J20" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K20" s="25" t="n">
+      <c r="K20" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L20" s="7" t="inlineStr">
@@ -6607,7 +6697,8 @@
         </is>
       </c>
       <c r="N20" s="7" t="inlineStr"/>
-      <c r="O20" s="7" t="inlineStr">
+      <c r="O20" s="7" t="inlineStr"/>
+      <c r="P20" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6629,7 +6720,7 @@
           <t>3763352</t>
         </is>
       </c>
-      <c r="D21" s="24" t="n">
+      <c r="D21" s="28" t="n">
         <v>45786</v>
       </c>
       <c r="E21" s="7" t="inlineStr">
@@ -6654,7 +6745,7 @@
       <c r="J21" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K21" s="25" t="n">
+      <c r="K21" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L21" s="7" t="inlineStr">
@@ -6668,7 +6759,8 @@
         </is>
       </c>
       <c r="N21" s="7" t="inlineStr"/>
-      <c r="O21" s="7" t="inlineStr">
+      <c r="O21" s="7" t="inlineStr"/>
+      <c r="P21" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6690,7 +6782,7 @@
           <t>3763352</t>
         </is>
       </c>
-      <c r="D22" s="24" t="n">
+      <c r="D22" s="28" t="n">
         <v>45786</v>
       </c>
       <c r="E22" s="7" t="inlineStr">
@@ -6715,7 +6807,7 @@
       <c r="J22" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K22" s="25" t="n">
+      <c r="K22" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L22" s="7" t="inlineStr">
@@ -6729,7 +6821,8 @@
         </is>
       </c>
       <c r="N22" s="7" t="inlineStr"/>
-      <c r="O22" s="7" t="inlineStr">
+      <c r="O22" s="7" t="inlineStr"/>
+      <c r="P22" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6751,7 +6844,7 @@
           <t>3763351</t>
         </is>
       </c>
-      <c r="D23" s="24" t="n">
+      <c r="D23" s="28" t="n">
         <v>45786</v>
       </c>
       <c r="E23" s="7" t="inlineStr">
@@ -6776,7 +6869,7 @@
       <c r="J23" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K23" s="25" t="n">
+      <c r="K23" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L23" s="7" t="inlineStr">
@@ -6790,7 +6883,8 @@
         </is>
       </c>
       <c r="N23" s="7" t="inlineStr"/>
-      <c r="O23" s="7" t="inlineStr">
+      <c r="O23" s="7" t="inlineStr"/>
+      <c r="P23" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6812,7 +6906,7 @@
           <t>3763351</t>
         </is>
       </c>
-      <c r="D24" s="24" t="n">
+      <c r="D24" s="28" t="n">
         <v>45786</v>
       </c>
       <c r="E24" s="7" t="inlineStr">
@@ -6837,7 +6931,7 @@
       <c r="J24" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K24" s="25" t="n">
+      <c r="K24" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L24" s="7" t="inlineStr">
@@ -6851,7 +6945,8 @@
         </is>
       </c>
       <c r="N24" s="7" t="inlineStr"/>
-      <c r="O24" s="7" t="inlineStr">
+      <c r="O24" s="7" t="inlineStr"/>
+      <c r="P24" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6873,7 +6968,7 @@
           <t>3763352</t>
         </is>
       </c>
-      <c r="D25" s="24" t="n">
+      <c r="D25" s="28" t="n">
         <v>45786</v>
       </c>
       <c r="E25" s="7" t="inlineStr">
@@ -6898,7 +6993,7 @@
       <c r="J25" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K25" s="25" t="n">
+      <c r="K25" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L25" s="7" t="inlineStr">
@@ -6912,7 +7007,8 @@
         </is>
       </c>
       <c r="N25" s="7" t="inlineStr"/>
-      <c r="O25" s="7" t="inlineStr">
+      <c r="O25" s="7" t="inlineStr"/>
+      <c r="P25" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6934,7 +7030,7 @@
           <t>3763352</t>
         </is>
       </c>
-      <c r="D26" s="24" t="n">
+      <c r="D26" s="28" t="n">
         <v>45786</v>
       </c>
       <c r="E26" s="7" t="inlineStr">
@@ -6959,7 +7055,7 @@
       <c r="J26" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K26" s="25" t="n">
+      <c r="K26" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L26" s="7" t="inlineStr">
@@ -6973,7 +7069,8 @@
         </is>
       </c>
       <c r="N26" s="7" t="inlineStr"/>
-      <c r="O26" s="7" t="inlineStr">
+      <c r="O26" s="7" t="inlineStr"/>
+      <c r="P26" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -6995,7 +7092,7 @@
           <t>3763656</t>
         </is>
       </c>
-      <c r="D27" s="24" t="n">
+      <c r="D27" s="28" t="n">
         <v>45792</v>
       </c>
       <c r="E27" s="7" t="inlineStr">
@@ -7020,7 +7117,7 @@
       <c r="J27" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K27" s="25" t="n">
+      <c r="K27" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L27" s="7" t="inlineStr">
@@ -7034,7 +7131,8 @@
         </is>
       </c>
       <c r="N27" s="7" t="inlineStr"/>
-      <c r="O27" s="7" t="inlineStr">
+      <c r="O27" s="7" t="inlineStr"/>
+      <c r="P27" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7056,7 +7154,7 @@
           <t>3763657</t>
         </is>
       </c>
-      <c r="D28" s="24" t="n">
+      <c r="D28" s="28" t="n">
         <v>45792</v>
       </c>
       <c r="E28" s="7" t="inlineStr">
@@ -7081,7 +7179,7 @@
       <c r="J28" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K28" s="25" t="n">
+      <c r="K28" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L28" s="7" t="inlineStr">
@@ -7095,7 +7193,8 @@
         </is>
       </c>
       <c r="N28" s="7" t="inlineStr"/>
-      <c r="O28" s="7" t="inlineStr">
+      <c r="O28" s="7" t="inlineStr"/>
+      <c r="P28" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7117,7 +7216,7 @@
           <t>3763657</t>
         </is>
       </c>
-      <c r="D29" s="24" t="n">
+      <c r="D29" s="28" t="n">
         <v>45792</v>
       </c>
       <c r="E29" s="7" t="inlineStr">
@@ -7142,7 +7241,7 @@
       <c r="J29" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K29" s="25" t="n">
+      <c r="K29" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L29" s="7" t="inlineStr">
@@ -7156,7 +7255,8 @@
         </is>
       </c>
       <c r="N29" s="7" t="inlineStr"/>
-      <c r="O29" s="7" t="inlineStr">
+      <c r="O29" s="7" t="inlineStr"/>
+      <c r="P29" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7178,7 +7278,7 @@
           <t>3763656</t>
         </is>
       </c>
-      <c r="D30" s="24" t="n">
+      <c r="D30" s="28" t="n">
         <v>45792</v>
       </c>
       <c r="E30" s="7" t="inlineStr">
@@ -7203,7 +7303,7 @@
       <c r="J30" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K30" s="25" t="n">
+      <c r="K30" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L30" s="7" t="inlineStr">
@@ -7217,7 +7317,8 @@
         </is>
       </c>
       <c r="N30" s="7" t="inlineStr"/>
-      <c r="O30" s="7" t="inlineStr">
+      <c r="O30" s="7" t="inlineStr"/>
+      <c r="P30" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7239,7 +7340,7 @@
           <t>3763658</t>
         </is>
       </c>
-      <c r="D31" s="24" t="n">
+      <c r="D31" s="28" t="n">
         <v>45793</v>
       </c>
       <c r="E31" s="7" t="inlineStr">
@@ -7264,7 +7365,7 @@
       <c r="J31" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K31" s="25" t="n">
+      <c r="K31" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L31" s="7" t="inlineStr">
@@ -7278,7 +7379,8 @@
         </is>
       </c>
       <c r="N31" s="7" t="inlineStr"/>
-      <c r="O31" s="7" t="inlineStr">
+      <c r="O31" s="7" t="inlineStr"/>
+      <c r="P31" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7300,7 +7402,7 @@
           <t>3763658</t>
         </is>
       </c>
-      <c r="D32" s="24" t="n">
+      <c r="D32" s="28" t="n">
         <v>45793</v>
       </c>
       <c r="E32" s="7" t="inlineStr">
@@ -7325,7 +7427,7 @@
       <c r="J32" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K32" s="25" t="n">
+      <c r="K32" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L32" s="7" t="inlineStr">
@@ -7339,7 +7441,8 @@
         </is>
       </c>
       <c r="N32" s="7" t="inlineStr"/>
-      <c r="O32" s="7" t="inlineStr">
+      <c r="O32" s="7" t="inlineStr"/>
+      <c r="P32" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7361,7 +7464,7 @@
           <t>3765098</t>
         </is>
       </c>
-      <c r="D33" s="24" t="n">
+      <c r="D33" s="28" t="n">
         <v>45799</v>
       </c>
       <c r="E33" s="7" t="inlineStr">
@@ -7386,7 +7489,7 @@
       <c r="J33" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K33" s="25" t="n">
+      <c r="K33" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L33" s="7" t="inlineStr">
@@ -7400,7 +7503,8 @@
         </is>
       </c>
       <c r="N33" s="7" t="inlineStr"/>
-      <c r="O33" s="7" t="inlineStr">
+      <c r="O33" s="7" t="inlineStr"/>
+      <c r="P33" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7422,7 +7526,7 @@
           <t>3765098</t>
         </is>
       </c>
-      <c r="D34" s="24" t="n">
+      <c r="D34" s="28" t="n">
         <v>45799</v>
       </c>
       <c r="E34" s="7" t="inlineStr">
@@ -7447,7 +7551,7 @@
       <c r="J34" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K34" s="25" t="n">
+      <c r="K34" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L34" s="7" t="inlineStr">
@@ -7461,7 +7565,8 @@
         </is>
       </c>
       <c r="N34" s="7" t="inlineStr"/>
-      <c r="O34" s="7" t="inlineStr">
+      <c r="O34" s="7" t="inlineStr"/>
+      <c r="P34" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7483,7 +7588,7 @@
           <t>3761902</t>
         </is>
       </c>
-      <c r="D35" s="24" t="n">
+      <c r="D35" s="28" t="n">
         <v>45779</v>
       </c>
       <c r="E35" s="7" t="inlineStr">
@@ -7508,7 +7613,7 @@
       <c r="J35" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K35" s="25" t="n">
+      <c r="K35" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L35" s="7" t="inlineStr">
@@ -7522,7 +7627,8 @@
         </is>
       </c>
       <c r="N35" s="7" t="inlineStr"/>
-      <c r="O35" s="7" t="inlineStr">
+      <c r="O35" s="7" t="inlineStr"/>
+      <c r="P35" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7544,7 +7650,7 @@
           <t>3761902</t>
         </is>
       </c>
-      <c r="D36" s="24" t="n">
+      <c r="D36" s="28" t="n">
         <v>45779</v>
       </c>
       <c r="E36" s="7" t="inlineStr">
@@ -7569,7 +7675,7 @@
       <c r="J36" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K36" s="25" t="n">
+      <c r="K36" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L36" s="7" t="inlineStr">
@@ -7583,7 +7689,8 @@
         </is>
       </c>
       <c r="N36" s="7" t="inlineStr"/>
-      <c r="O36" s="7" t="inlineStr">
+      <c r="O36" s="7" t="inlineStr"/>
+      <c r="P36" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7605,7 +7712,7 @@
           <t>3765099</t>
         </is>
       </c>
-      <c r="D37" s="24" t="n">
+      <c r="D37" s="28" t="n">
         <v>45800</v>
       </c>
       <c r="E37" s="7" t="inlineStr">
@@ -7630,7 +7737,7 @@
       <c r="J37" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K37" s="25" t="n">
+      <c r="K37" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L37" s="7" t="inlineStr">
@@ -7644,7 +7751,8 @@
         </is>
       </c>
       <c r="N37" s="7" t="inlineStr"/>
-      <c r="O37" s="7" t="inlineStr">
+      <c r="O37" s="7" t="inlineStr"/>
+      <c r="P37" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7666,7 +7774,7 @@
           <t>3765099</t>
         </is>
       </c>
-      <c r="D38" s="24" t="n">
+      <c r="D38" s="28" t="n">
         <v>45800</v>
       </c>
       <c r="E38" s="7" t="inlineStr">
@@ -7691,7 +7799,7 @@
       <c r="J38" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K38" s="25" t="n">
+      <c r="K38" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L38" s="7" t="inlineStr">
@@ -7705,7 +7813,8 @@
         </is>
       </c>
       <c r="N38" s="7" t="inlineStr"/>
-      <c r="O38" s="7" t="inlineStr">
+      <c r="O38" s="7" t="inlineStr"/>
+      <c r="P38" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7727,7 +7836,7 @@
           <t>3767326</t>
         </is>
       </c>
-      <c r="D39" s="24" t="n">
+      <c r="D39" s="28" t="n">
         <v>45813</v>
       </c>
       <c r="E39" s="7" t="inlineStr">
@@ -7752,7 +7861,7 @@
       <c r="J39" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K39" s="25" t="n">
+      <c r="K39" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L39" s="7" t="inlineStr">
@@ -7766,7 +7875,8 @@
         </is>
       </c>
       <c r="N39" s="7" t="inlineStr"/>
-      <c r="O39" s="7" t="inlineStr">
+      <c r="O39" s="7" t="inlineStr"/>
+      <c r="P39" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7788,7 +7898,7 @@
           <t>3766901</t>
         </is>
       </c>
-      <c r="D40" s="24" t="n">
+      <c r="D40" s="28" t="n">
         <v>45805</v>
       </c>
       <c r="E40" s="7" t="inlineStr">
@@ -7813,7 +7923,7 @@
       <c r="J40" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K40" s="25" t="n">
+      <c r="K40" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L40" s="7" t="inlineStr">
@@ -7823,7 +7933,8 @@
       </c>
       <c r="M40" s="7" t="inlineStr"/>
       <c r="N40" s="7" t="inlineStr"/>
-      <c r="O40" s="7" t="inlineStr">
+      <c r="O40" s="7" t="inlineStr"/>
+      <c r="P40" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7845,7 +7956,7 @@
           <t>3767326</t>
         </is>
       </c>
-      <c r="D41" s="24" t="n">
+      <c r="D41" s="28" t="n">
         <v>45813</v>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -7870,7 +7981,7 @@
       <c r="J41" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K41" s="25" t="n">
+      <c r="K41" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L41" s="7" t="inlineStr">
@@ -7884,7 +7995,8 @@
         </is>
       </c>
       <c r="N41" s="7" t="inlineStr"/>
-      <c r="O41" s="7" t="inlineStr">
+      <c r="O41" s="7" t="inlineStr"/>
+      <c r="P41" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7906,7 +8018,7 @@
           <t>3767326</t>
         </is>
       </c>
-      <c r="D42" s="24" t="n">
+      <c r="D42" s="28" t="n">
         <v>45813</v>
       </c>
       <c r="E42" s="7" t="inlineStr">
@@ -7931,7 +8043,7 @@
       <c r="J42" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K42" s="25" t="n">
+      <c r="K42" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L42" s="7" t="inlineStr">
@@ -7945,7 +8057,8 @@
         </is>
       </c>
       <c r="N42" s="7" t="inlineStr"/>
-      <c r="O42" s="7" t="inlineStr">
+      <c r="O42" s="7" t="inlineStr"/>
+      <c r="P42" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -7967,7 +8080,7 @@
           <t>3767326</t>
         </is>
       </c>
-      <c r="D43" s="24" t="n">
+      <c r="D43" s="28" t="n">
         <v>45813</v>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -7992,7 +8105,7 @@
       <c r="J43" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K43" s="25" t="n">
+      <c r="K43" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L43" s="7" t="inlineStr">
@@ -8006,7 +8119,8 @@
         </is>
       </c>
       <c r="N43" s="7" t="inlineStr"/>
-      <c r="O43" s="7" t="inlineStr">
+      <c r="O43" s="7" t="inlineStr"/>
+      <c r="P43" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8028,7 +8142,7 @@
           <t>3767326</t>
         </is>
       </c>
-      <c r="D44" s="24" t="n">
+      <c r="D44" s="28" t="n">
         <v>45813</v>
       </c>
       <c r="E44" s="7" t="inlineStr">
@@ -8053,7 +8167,7 @@
       <c r="J44" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K44" s="25" t="n">
+      <c r="K44" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L44" s="7" t="inlineStr">
@@ -8067,7 +8181,8 @@
         </is>
       </c>
       <c r="N44" s="7" t="inlineStr"/>
-      <c r="O44" s="7" t="inlineStr">
+      <c r="O44" s="7" t="inlineStr"/>
+      <c r="P44" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8089,7 +8204,7 @@
           <t>3767327</t>
         </is>
       </c>
-      <c r="D45" s="24" t="n">
+      <c r="D45" s="28" t="n">
         <v>45814</v>
       </c>
       <c r="E45" s="7" t="inlineStr">
@@ -8114,7 +8229,7 @@
       <c r="J45" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K45" s="25" t="n">
+      <c r="K45" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L45" s="7" t="inlineStr">
@@ -8124,7 +8239,8 @@
       </c>
       <c r="M45" s="7" t="inlineStr"/>
       <c r="N45" s="7" t="inlineStr"/>
-      <c r="O45" s="7" t="inlineStr">
+      <c r="O45" s="7" t="inlineStr"/>
+      <c r="P45" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8146,7 +8262,7 @@
           <t>3768779</t>
         </is>
       </c>
-      <c r="D46" s="24" t="n">
+      <c r="D46" s="28" t="n">
         <v>45821</v>
       </c>
       <c r="E46" s="7" t="inlineStr">
@@ -8171,7 +8287,7 @@
       <c r="J46" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K46" s="25" t="n">
+      <c r="K46" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L46" s="7" t="inlineStr">
@@ -8185,7 +8301,8 @@
         </is>
       </c>
       <c r="N46" s="7" t="inlineStr"/>
-      <c r="O46" s="7" t="inlineStr">
+      <c r="O46" s="7" t="inlineStr"/>
+      <c r="P46" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8207,7 +8324,7 @@
           <t>3768778</t>
         </is>
       </c>
-      <c r="D47" s="24" t="n">
+      <c r="D47" s="28" t="n">
         <v>45821</v>
       </c>
       <c r="E47" s="7" t="inlineStr">
@@ -8232,7 +8349,7 @@
       <c r="J47" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K47" s="25" t="n">
+      <c r="K47" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L47" s="7" t="inlineStr">
@@ -8246,7 +8363,8 @@
         </is>
       </c>
       <c r="N47" s="7" t="inlineStr"/>
-      <c r="O47" s="7" t="inlineStr">
+      <c r="O47" s="7" t="inlineStr"/>
+      <c r="P47" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8268,7 +8386,7 @@
           <t>3768779</t>
         </is>
       </c>
-      <c r="D48" s="24" t="n">
+      <c r="D48" s="28" t="n">
         <v>45821</v>
       </c>
       <c r="E48" s="7" t="inlineStr">
@@ -8293,7 +8411,7 @@
       <c r="J48" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K48" s="25" t="n">
+      <c r="K48" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L48" s="7" t="inlineStr">
@@ -8307,7 +8425,8 @@
         </is>
       </c>
       <c r="N48" s="7" t="inlineStr"/>
-      <c r="O48" s="7" t="inlineStr">
+      <c r="O48" s="7" t="inlineStr"/>
+      <c r="P48" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8329,7 +8448,7 @@
           <t>3768778</t>
         </is>
       </c>
-      <c r="D49" s="24" t="n">
+      <c r="D49" s="28" t="n">
         <v>45821</v>
       </c>
       <c r="E49" s="7" t="inlineStr">
@@ -8354,7 +8473,7 @@
       <c r="J49" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K49" s="25" t="n">
+      <c r="K49" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L49" s="7" t="inlineStr">
@@ -8368,7 +8487,8 @@
         </is>
       </c>
       <c r="N49" s="7" t="inlineStr"/>
-      <c r="O49" s="7" t="inlineStr">
+      <c r="O49" s="7" t="inlineStr"/>
+      <c r="P49" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8390,7 +8510,7 @@
           <t>3768778</t>
         </is>
       </c>
-      <c r="D50" s="24" t="n">
+      <c r="D50" s="28" t="n">
         <v>45821</v>
       </c>
       <c r="E50" s="7" t="inlineStr">
@@ -8415,7 +8535,7 @@
       <c r="J50" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K50" s="25" t="n">
+      <c r="K50" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L50" s="7" t="inlineStr">
@@ -8429,7 +8549,8 @@
         </is>
       </c>
       <c r="N50" s="7" t="inlineStr"/>
-      <c r="O50" s="7" t="inlineStr">
+      <c r="O50" s="7" t="inlineStr"/>
+      <c r="P50" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8451,7 +8572,7 @@
           <t>3768386</t>
         </is>
       </c>
-      <c r="D51" s="24" t="n">
+      <c r="D51" s="28" t="n">
         <v>45824</v>
       </c>
       <c r="E51" s="7" t="inlineStr">
@@ -8476,7 +8597,7 @@
       <c r="J51" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K51" s="25" t="n">
+      <c r="K51" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L51" s="7" t="inlineStr">
@@ -8486,7 +8607,8 @@
       </c>
       <c r="M51" s="7" t="inlineStr"/>
       <c r="N51" s="7" t="inlineStr"/>
-      <c r="O51" s="7" t="inlineStr">
+      <c r="O51" s="7" t="inlineStr"/>
+      <c r="P51" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8508,7 +8630,7 @@
           <t>3767326</t>
         </is>
       </c>
-      <c r="D52" s="24" t="n">
+      <c r="D52" s="28" t="n">
         <v>45813</v>
       </c>
       <c r="E52" s="7" t="inlineStr">
@@ -8533,7 +8655,7 @@
       <c r="J52" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K52" s="25" t="n">
+      <c r="K52" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L52" s="7" t="inlineStr">
@@ -8547,7 +8669,8 @@
         </is>
       </c>
       <c r="N52" s="7" t="inlineStr"/>
-      <c r="O52" s="7" t="inlineStr">
+      <c r="O52" s="7" t="inlineStr"/>
+      <c r="P52" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8569,7 +8692,7 @@
           <t>3769256</t>
         </is>
       </c>
-      <c r="D53" s="24" t="n">
+      <c r="D53" s="28" t="n">
         <v>45828</v>
       </c>
       <c r="E53" s="7" t="inlineStr">
@@ -8594,7 +8717,7 @@
       <c r="J53" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K53" s="25" t="n">
+      <c r="K53" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L53" s="7" t="inlineStr">
@@ -8608,7 +8731,8 @@
         </is>
       </c>
       <c r="N53" s="7" t="inlineStr"/>
-      <c r="O53" s="7" t="inlineStr">
+      <c r="O53" s="7" t="inlineStr"/>
+      <c r="P53" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8630,7 +8754,7 @@
           <t>3769256</t>
         </is>
       </c>
-      <c r="D54" s="24" t="n">
+      <c r="D54" s="28" t="n">
         <v>45828</v>
       </c>
       <c r="E54" s="7" t="inlineStr">
@@ -8655,7 +8779,7 @@
       <c r="J54" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K54" s="25" t="n">
+      <c r="K54" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L54" s="7" t="inlineStr">
@@ -8669,7 +8793,8 @@
         </is>
       </c>
       <c r="N54" s="7" t="inlineStr"/>
-      <c r="O54" s="7" t="inlineStr">
+      <c r="O54" s="7" t="inlineStr"/>
+      <c r="P54" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8691,7 +8816,7 @@
           <t>3769255</t>
         </is>
       </c>
-      <c r="D55" s="24" t="n">
+      <c r="D55" s="28" t="n">
         <v>45828</v>
       </c>
       <c r="E55" s="7" t="inlineStr">
@@ -8716,7 +8841,7 @@
       <c r="J55" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K55" s="25" t="n">
+      <c r="K55" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L55" s="7" t="inlineStr">
@@ -8730,7 +8855,8 @@
         </is>
       </c>
       <c r="N55" s="7" t="inlineStr"/>
-      <c r="O55" s="7" t="inlineStr">
+      <c r="O55" s="7" t="inlineStr"/>
+      <c r="P55" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8752,7 +8878,7 @@
           <t>3769256</t>
         </is>
       </c>
-      <c r="D56" s="24" t="n">
+      <c r="D56" s="28" t="n">
         <v>45828</v>
       </c>
       <c r="E56" s="7" t="inlineStr">
@@ -8777,7 +8903,7 @@
       <c r="J56" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K56" s="25" t="n">
+      <c r="K56" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L56" s="7" t="inlineStr">
@@ -8791,7 +8917,8 @@
         </is>
       </c>
       <c r="N56" s="7" t="inlineStr"/>
-      <c r="O56" s="7" t="inlineStr">
+      <c r="O56" s="7" t="inlineStr"/>
+      <c r="P56" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8813,7 +8940,7 @@
           <t>3770616</t>
         </is>
       </c>
-      <c r="D57" s="24" t="n">
+      <c r="D57" s="28" t="n">
         <v>45834</v>
       </c>
       <c r="E57" s="7" t="inlineStr">
@@ -8838,7 +8965,7 @@
       <c r="J57" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K57" s="25" t="n">
+      <c r="K57" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L57" s="7" t="inlineStr">
@@ -8852,7 +8979,8 @@
         </is>
       </c>
       <c r="N57" s="7" t="inlineStr"/>
-      <c r="O57" s="7" t="inlineStr">
+      <c r="O57" s="7" t="inlineStr"/>
+      <c r="P57" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8874,7 +9002,7 @@
           <t>3770616</t>
         </is>
       </c>
-      <c r="D58" s="24" t="n">
+      <c r="D58" s="28" t="n">
         <v>45834</v>
       </c>
       <c r="E58" s="7" t="inlineStr">
@@ -8899,7 +9027,7 @@
       <c r="J58" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K58" s="25" t="n">
+      <c r="K58" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L58" s="7" t="inlineStr">
@@ -8913,7 +9041,8 @@
         </is>
       </c>
       <c r="N58" s="7" t="inlineStr"/>
-      <c r="O58" s="7" t="inlineStr">
+      <c r="O58" s="7" t="inlineStr"/>
+      <c r="P58" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8935,7 +9064,7 @@
           <t>3770617</t>
         </is>
       </c>
-      <c r="D59" s="24" t="n">
+      <c r="D59" s="28" t="n">
         <v>45835</v>
       </c>
       <c r="E59" s="7" t="inlineStr">
@@ -8960,7 +9089,7 @@
       <c r="J59" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K59" s="25" t="n">
+      <c r="K59" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L59" s="7" t="inlineStr">
@@ -8974,7 +9103,8 @@
         </is>
       </c>
       <c r="N59" s="7" t="inlineStr"/>
-      <c r="O59" s="7" t="inlineStr">
+      <c r="O59" s="7" t="inlineStr"/>
+      <c r="P59" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -8996,7 +9126,7 @@
           <t>3770617</t>
         </is>
       </c>
-      <c r="D60" s="24" t="n">
+      <c r="D60" s="28" t="n">
         <v>45835</v>
       </c>
       <c r="E60" s="7" t="inlineStr">
@@ -9021,7 +9151,7 @@
       <c r="J60" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K60" s="25" t="n">
+      <c r="K60" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L60" s="7" t="inlineStr">
@@ -9035,7 +9165,8 @@
         </is>
       </c>
       <c r="N60" s="7" t="inlineStr"/>
-      <c r="O60" s="7" t="inlineStr">
+      <c r="O60" s="7" t="inlineStr"/>
+      <c r="P60" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -9057,7 +9188,7 @@
           <t>3770617</t>
         </is>
       </c>
-      <c r="D61" s="24" t="n">
+      <c r="D61" s="28" t="n">
         <v>45835</v>
       </c>
       <c r="E61" s="7" t="inlineStr">
@@ -9082,7 +9213,7 @@
       <c r="J61" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K61" s="25" t="n">
+      <c r="K61" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L61" s="7" t="inlineStr">
@@ -9096,7 +9227,8 @@
         </is>
       </c>
       <c r="N61" s="7" t="inlineStr"/>
-      <c r="O61" s="7" t="inlineStr">
+      <c r="O61" s="7" t="inlineStr"/>
+      <c r="P61" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -9118,7 +9250,7 @@
           <t>3770617</t>
         </is>
       </c>
-      <c r="D62" s="24" t="n">
+      <c r="D62" s="28" t="n">
         <v>45835</v>
       </c>
       <c r="E62" s="7" t="inlineStr">
@@ -9143,7 +9275,7 @@
       <c r="J62" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K62" s="25" t="n">
+      <c r="K62" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L62" s="7" t="inlineStr">
@@ -9157,7 +9289,8 @@
         </is>
       </c>
       <c r="N62" s="7" t="inlineStr"/>
-      <c r="O62" s="7" t="inlineStr">
+      <c r="O62" s="7" t="inlineStr"/>
+      <c r="P62" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -9179,7 +9312,7 @@
           <t>3771714</t>
         </is>
       </c>
-      <c r="D63" s="24" t="n">
+      <c r="D63" s="28" t="n">
         <v>45841</v>
       </c>
       <c r="E63" s="7" t="inlineStr">
@@ -9204,7 +9337,7 @@
       <c r="J63" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K63" s="25" t="n">
+      <c r="K63" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L63" s="7" t="inlineStr">
@@ -9218,7 +9351,8 @@
         </is>
       </c>
       <c r="N63" s="7" t="inlineStr"/>
-      <c r="O63" s="7" t="inlineStr">
+      <c r="O63" s="7" t="inlineStr"/>
+      <c r="P63" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -9240,7 +9374,7 @@
           <t>3771714</t>
         </is>
       </c>
-      <c r="D64" s="24" t="n">
+      <c r="D64" s="28" t="n">
         <v>45841</v>
       </c>
       <c r="E64" s="7" t="inlineStr">
@@ -9265,7 +9399,7 @@
       <c r="J64" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K64" s="25" t="n">
+      <c r="K64" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L64" s="7" t="inlineStr">
@@ -9279,7 +9413,8 @@
         </is>
       </c>
       <c r="N64" s="7" t="inlineStr"/>
-      <c r="O64" s="7" t="inlineStr">
+      <c r="O64" s="7" t="inlineStr"/>
+      <c r="P64" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -9301,7 +9436,7 @@
           <t>3771714</t>
         </is>
       </c>
-      <c r="D65" s="24" t="n">
+      <c r="D65" s="28" t="n">
         <v>45841</v>
       </c>
       <c r="E65" s="7" t="inlineStr">
@@ -9326,7 +9461,7 @@
       <c r="J65" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K65" s="25" t="n">
+      <c r="K65" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L65" s="7" t="inlineStr">
@@ -9340,7 +9475,8 @@
         </is>
       </c>
       <c r="N65" s="7" t="inlineStr"/>
-      <c r="O65" s="7" t="inlineStr">
+      <c r="O65" s="7" t="inlineStr"/>
+      <c r="P65" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -9362,7 +9498,7 @@
           <t>3771715</t>
         </is>
       </c>
-      <c r="D66" s="24" t="n">
+      <c r="D66" s="28" t="n">
         <v>45842</v>
       </c>
       <c r="E66" s="7" t="inlineStr">
@@ -9387,7 +9523,7 @@
       <c r="J66" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K66" s="25" t="n">
+      <c r="K66" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L66" s="7" t="inlineStr">
@@ -9401,7 +9537,8 @@
         </is>
       </c>
       <c r="N66" s="7" t="inlineStr"/>
-      <c r="O66" s="7" t="inlineStr">
+      <c r="O66" s="7" t="inlineStr"/>
+      <c r="P66" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -9423,7 +9560,7 @@
           <t>3771715</t>
         </is>
       </c>
-      <c r="D67" s="24" t="n">
+      <c r="D67" s="28" t="n">
         <v>45842</v>
       </c>
       <c r="E67" s="7" t="inlineStr">
@@ -9448,7 +9585,7 @@
       <c r="J67" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K67" s="25" t="n">
+      <c r="K67" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L67" s="7" t="inlineStr">
@@ -9462,7 +9599,8 @@
         </is>
       </c>
       <c r="N67" s="7" t="inlineStr"/>
-      <c r="O67" s="7" t="inlineStr">
+      <c r="O67" s="7" t="inlineStr"/>
+      <c r="P67" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -9484,7 +9622,7 @@
           <t>3769255</t>
         </is>
       </c>
-      <c r="D68" s="24" t="n">
+      <c r="D68" s="28" t="n">
         <v>45828</v>
       </c>
       <c r="E68" s="7" t="inlineStr">
@@ -9509,7 +9647,7 @@
       <c r="J68" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K68" s="25" t="n">
+      <c r="K68" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L68" s="7" t="inlineStr">
@@ -9523,70 +9661,76 @@
         </is>
       </c>
       <c r="N68" s="7" t="inlineStr"/>
-      <c r="O68" s="7" t="inlineStr">
+      <c r="O68" s="7" t="inlineStr"/>
+      <c r="P68" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
       </c>
     </row>
     <row r="69">
-      <c r="A69" s="7" t="inlineStr">
+      <c r="A69" s="20" t="inlineStr">
         <is>
           <t>32921515</t>
         </is>
       </c>
-      <c r="B69" s="7" t="inlineStr">
+      <c r="B69" s="20" t="inlineStr">
         <is>
           <t>3771715</t>
         </is>
       </c>
-      <c r="C69" s="7" t="inlineStr">
+      <c r="C69" s="20" t="inlineStr">
         <is>
           <t>3771715</t>
         </is>
       </c>
-      <c r="D69" s="24" t="n">
+      <c r="D69" s="21" t="n">
         <v>45842</v>
       </c>
-      <c r="E69" s="7" t="inlineStr">
-        <is>
-          <t>GR</t>
-        </is>
-      </c>
-      <c r="F69" s="7" t="inlineStr">
+      <c r="E69" s="20" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+      <c r="F69" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">57300    </t>
         </is>
       </c>
-      <c r="G69" s="7" t="n">
+      <c r="G69" s="20" t="n">
         <v>5886</v>
       </c>
-      <c r="H69" s="10" t="n">
+      <c r="H69" s="22" t="n">
         <v>1921.6</v>
       </c>
-      <c r="I69" s="10" t="n">
+      <c r="I69" s="22" t="n">
         <v>1921.6</v>
       </c>
-      <c r="J69" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K69" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L69" s="7" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="M69" s="7" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="N69" s="7" t="inlineStr"/>
-      <c r="O69" s="7" t="inlineStr">
-        <is>
-          <t>±5%</t>
+      <c r="J69" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K69" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L69" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M69" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="N69" s="20" t="inlineStr"/>
+      <c r="O69" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="P69" s="20" t="inlineStr">
+        <is>
+          <t>Multi-Row</t>
         </is>
       </c>
     </row>
@@ -9606,7 +9750,7 @@
           <t>3772453</t>
         </is>
       </c>
-      <c r="D70" s="24" t="n">
+      <c r="D70" s="28" t="n">
         <v>45848</v>
       </c>
       <c r="E70" s="7" t="inlineStr">
@@ -9631,7 +9775,7 @@
       <c r="J70" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K70" s="25" t="n">
+      <c r="K70" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L70" s="7" t="inlineStr">
@@ -9645,7 +9789,8 @@
         </is>
       </c>
       <c r="N70" s="7" t="inlineStr"/>
-      <c r="O70" s="7" t="inlineStr">
+      <c r="O70" s="7" t="inlineStr"/>
+      <c r="P70" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -9667,7 +9812,7 @@
           <t>3772453</t>
         </is>
       </c>
-      <c r="D71" s="24" t="n">
+      <c r="D71" s="28" t="n">
         <v>45848</v>
       </c>
       <c r="E71" s="7" t="inlineStr">
@@ -9692,7 +9837,7 @@
       <c r="J71" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K71" s="25" t="n">
+      <c r="K71" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L71" s="7" t="inlineStr">
@@ -9706,192 +9851,208 @@
         </is>
       </c>
       <c r="N71" s="7" t="inlineStr"/>
-      <c r="O71" s="7" t="inlineStr">
+      <c r="O71" s="7" t="inlineStr"/>
+      <c r="P71" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
       </c>
     </row>
     <row r="72">
-      <c r="A72" s="7" t="inlineStr">
+      <c r="A72" s="20" t="inlineStr">
         <is>
           <t>32925053</t>
         </is>
       </c>
-      <c r="B72" s="7" t="inlineStr">
+      <c r="B72" s="20" t="inlineStr">
         <is>
           <t>3772453</t>
         </is>
       </c>
-      <c r="C72" s="7" t="inlineStr">
+      <c r="C72" s="20" t="inlineStr">
         <is>
           <t>3772453</t>
         </is>
       </c>
-      <c r="D72" s="24" t="n">
+      <c r="D72" s="21" t="n">
         <v>45848</v>
       </c>
-      <c r="E72" s="7" t="inlineStr">
-        <is>
-          <t>GR</t>
-        </is>
-      </c>
-      <c r="F72" s="7" t="inlineStr">
+      <c r="E72" s="20" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+      <c r="F72" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">23200    </t>
         </is>
       </c>
-      <c r="G72" s="7" t="n">
+      <c r="G72" s="20" t="n">
         <v>2068</v>
       </c>
-      <c r="H72" s="10" t="n">
+      <c r="H72" s="22" t="n">
         <v>352.01</v>
       </c>
-      <c r="I72" s="10" t="n">
+      <c r="I72" s="22" t="n">
         <v>352.01</v>
       </c>
-      <c r="J72" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K72" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L72" s="7" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="M72" s="7" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="N72" s="7" t="inlineStr"/>
-      <c r="O72" s="7" t="inlineStr">
-        <is>
-          <t>±5%</t>
+      <c r="J72" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K72" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L72" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M72" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="N72" s="20" t="inlineStr"/>
+      <c r="O72" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="P72" s="20" t="inlineStr">
+        <is>
+          <t>Multi-Row</t>
         </is>
       </c>
     </row>
     <row r="73">
-      <c r="A73" s="7" t="inlineStr">
+      <c r="A73" s="20" t="inlineStr">
         <is>
           <t>32925054</t>
         </is>
       </c>
-      <c r="B73" s="7" t="inlineStr">
+      <c r="B73" s="20" t="inlineStr">
         <is>
           <t>3772454</t>
         </is>
       </c>
-      <c r="C73" s="7" t="inlineStr">
+      <c r="C73" s="20" t="inlineStr">
         <is>
           <t>3772454</t>
         </is>
       </c>
-      <c r="D73" s="24" t="n">
+      <c r="D73" s="21" t="n">
         <v>45848</v>
       </c>
-      <c r="E73" s="7" t="inlineStr">
-        <is>
-          <t>GR</t>
-        </is>
-      </c>
-      <c r="F73" s="7" t="inlineStr">
+      <c r="E73" s="20" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+      <c r="F73" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">32011    </t>
         </is>
       </c>
-      <c r="G73" s="7" t="n">
+      <c r="G73" s="20" t="n">
         <v>1880</v>
       </c>
-      <c r="H73" s="10" t="n">
+      <c r="H73" s="22" t="n">
         <v>624.3099999999999</v>
       </c>
-      <c r="I73" s="10" t="n">
+      <c r="I73" s="22" t="n">
         <v>624.3099999999999</v>
       </c>
-      <c r="J73" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K73" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L73" s="7" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="M73" s="7" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="N73" s="7" t="inlineStr"/>
-      <c r="O73" s="7" t="inlineStr">
-        <is>
-          <t>±5%</t>
+      <c r="J73" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K73" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L73" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M73" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="N73" s="20" t="inlineStr"/>
+      <c r="O73" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="P73" s="20" t="inlineStr">
+        <is>
+          <t>Multi-Row</t>
         </is>
       </c>
     </row>
     <row r="74">
-      <c r="A74" s="7" t="inlineStr">
+      <c r="A74" s="20" t="inlineStr">
         <is>
           <t>32925056</t>
         </is>
       </c>
-      <c r="B74" s="7" t="inlineStr">
+      <c r="B74" s="20" t="inlineStr">
         <is>
           <t>3772453</t>
         </is>
       </c>
-      <c r="C74" s="7" t="inlineStr">
+      <c r="C74" s="20" t="inlineStr">
         <is>
           <t>3772453</t>
         </is>
       </c>
-      <c r="D74" s="24" t="n">
+      <c r="D74" s="21" t="n">
         <v>45848</v>
       </c>
-      <c r="E74" s="7" t="inlineStr">
-        <is>
-          <t>GR</t>
-        </is>
-      </c>
-      <c r="F74" s="7" t="inlineStr">
+      <c r="E74" s="20" t="inlineStr">
+        <is>
+          <t>GR</t>
+        </is>
+      </c>
+      <c r="F74" s="20" t="inlineStr">
         <is>
           <t xml:space="preserve">57001    </t>
         </is>
       </c>
-      <c r="G74" s="7" t="n">
+      <c r="G74" s="20" t="n">
         <v>9414</v>
       </c>
-      <c r="H74" s="10" t="n">
+      <c r="H74" s="22" t="n">
         <v>4233.61</v>
       </c>
-      <c r="I74" s="10" t="n">
+      <c r="I74" s="22" t="n">
         <v>4233.61</v>
       </c>
-      <c r="J74" s="10" t="n">
-        <v>0</v>
-      </c>
-      <c r="K74" s="25" t="n">
-        <v>0</v>
-      </c>
-      <c r="L74" s="7" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="M74" s="7" t="inlineStr">
-        <is>
-          <t>JA</t>
-        </is>
-      </c>
-      <c r="N74" s="7" t="inlineStr"/>
-      <c r="O74" s="7" t="inlineStr">
-        <is>
-          <t>±5%</t>
+      <c r="J74" s="22" t="n">
+        <v>0</v>
+      </c>
+      <c r="K74" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L74" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="M74" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="N74" s="20" t="inlineStr"/>
+      <c r="O74" s="20" t="inlineStr">
+        <is>
+          <t>JA</t>
+        </is>
+      </c>
+      <c r="P74" s="20" t="inlineStr">
+        <is>
+          <t>Multi-Row</t>
         </is>
       </c>
     </row>
@@ -9911,7 +10072,7 @@
           <t>3772453</t>
         </is>
       </c>
-      <c r="D75" s="24" t="n">
+      <c r="D75" s="28" t="n">
         <v>45848</v>
       </c>
       <c r="E75" s="7" t="inlineStr">
@@ -9936,7 +10097,7 @@
       <c r="J75" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K75" s="25" t="n">
+      <c r="K75" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L75" s="7" t="inlineStr">
@@ -9950,7 +10111,8 @@
         </is>
       </c>
       <c r="N75" s="7" t="inlineStr"/>
-      <c r="O75" s="7" t="inlineStr">
+      <c r="O75" s="7" t="inlineStr"/>
+      <c r="P75" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -9972,7 +10134,7 @@
           <t>3772454</t>
         </is>
       </c>
-      <c r="D76" s="24" t="n">
+      <c r="D76" s="28" t="n">
         <v>45848</v>
       </c>
       <c r="E76" s="7" t="inlineStr">
@@ -9997,7 +10159,7 @@
       <c r="J76" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K76" s="25" t="n">
+      <c r="K76" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L76" s="7" t="inlineStr">
@@ -10011,7 +10173,8 @@
         </is>
       </c>
       <c r="N76" s="7" t="inlineStr"/>
-      <c r="O76" s="7" t="inlineStr">
+      <c r="O76" s="7" t="inlineStr"/>
+      <c r="P76" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10033,7 +10196,7 @@
           <t>3774975</t>
         </is>
       </c>
-      <c r="D77" s="24" t="n">
+      <c r="D77" s="28" t="n">
         <v>45855</v>
       </c>
       <c r="E77" s="7" t="inlineStr">
@@ -10058,7 +10221,7 @@
       <c r="J77" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K77" s="25" t="n">
+      <c r="K77" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L77" s="7" t="inlineStr">
@@ -10072,7 +10235,8 @@
         </is>
       </c>
       <c r="N77" s="7" t="inlineStr"/>
-      <c r="O77" s="7" t="inlineStr">
+      <c r="O77" s="7" t="inlineStr"/>
+      <c r="P77" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10094,7 +10258,7 @@
           <t>3774975</t>
         </is>
       </c>
-      <c r="D78" s="24" t="n">
+      <c r="D78" s="28" t="n">
         <v>45855</v>
       </c>
       <c r="E78" s="7" t="inlineStr">
@@ -10119,7 +10283,7 @@
       <c r="J78" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K78" s="25" t="n">
+      <c r="K78" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L78" s="7" t="inlineStr">
@@ -10133,7 +10297,8 @@
         </is>
       </c>
       <c r="N78" s="7" t="inlineStr"/>
-      <c r="O78" s="7" t="inlineStr">
+      <c r="O78" s="7" t="inlineStr"/>
+      <c r="P78" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10155,7 +10320,7 @@
           <t>3774975</t>
         </is>
       </c>
-      <c r="D79" s="24" t="n">
+      <c r="D79" s="28" t="n">
         <v>45855</v>
       </c>
       <c r="E79" s="7" t="inlineStr">
@@ -10180,7 +10345,7 @@
       <c r="J79" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K79" s="25" t="n">
+      <c r="K79" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L79" s="7" t="inlineStr">
@@ -10194,7 +10359,8 @@
         </is>
       </c>
       <c r="N79" s="7" t="inlineStr"/>
-      <c r="O79" s="7" t="inlineStr">
+      <c r="O79" s="7" t="inlineStr"/>
+      <c r="P79" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10216,7 +10382,7 @@
           <t>3774975</t>
         </is>
       </c>
-      <c r="D80" s="24" t="n">
+      <c r="D80" s="28" t="n">
         <v>45855</v>
       </c>
       <c r="E80" s="7" t="inlineStr">
@@ -10241,7 +10407,7 @@
       <c r="J80" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K80" s="25" t="n">
+      <c r="K80" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L80" s="7" t="inlineStr">
@@ -10255,7 +10421,8 @@
         </is>
       </c>
       <c r="N80" s="7" t="inlineStr"/>
-      <c r="O80" s="7" t="inlineStr">
+      <c r="O80" s="7" t="inlineStr"/>
+      <c r="P80" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10277,7 +10444,7 @@
           <t>3774975</t>
         </is>
       </c>
-      <c r="D81" s="24" t="n">
+      <c r="D81" s="28" t="n">
         <v>45855</v>
       </c>
       <c r="E81" s="7" t="inlineStr">
@@ -10302,7 +10469,7 @@
       <c r="J81" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K81" s="25" t="n">
+      <c r="K81" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L81" s="7" t="inlineStr">
@@ -10316,7 +10483,8 @@
         </is>
       </c>
       <c r="N81" s="7" t="inlineStr"/>
-      <c r="O81" s="7" t="inlineStr">
+      <c r="O81" s="7" t="inlineStr"/>
+      <c r="P81" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10338,7 +10506,7 @@
           <t>3774975</t>
         </is>
       </c>
-      <c r="D82" s="24" t="n">
+      <c r="D82" s="28" t="n">
         <v>45855</v>
       </c>
       <c r="E82" s="7" t="inlineStr">
@@ -10363,7 +10531,7 @@
       <c r="J82" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K82" s="25" t="n">
+      <c r="K82" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L82" s="7" t="inlineStr">
@@ -10377,7 +10545,8 @@
         </is>
       </c>
       <c r="N82" s="7" t="inlineStr"/>
-      <c r="O82" s="7" t="inlineStr">
+      <c r="O82" s="7" t="inlineStr"/>
+      <c r="P82" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10399,7 +10568,7 @@
           <t>3774975</t>
         </is>
       </c>
-      <c r="D83" s="24" t="n">
+      <c r="D83" s="28" t="n">
         <v>45855</v>
       </c>
       <c r="E83" s="7" t="inlineStr">
@@ -10424,7 +10593,7 @@
       <c r="J83" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K83" s="25" t="n">
+      <c r="K83" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L83" s="7" t="inlineStr">
@@ -10438,7 +10607,8 @@
         </is>
       </c>
       <c r="N83" s="7" t="inlineStr"/>
-      <c r="O83" s="7" t="inlineStr">
+      <c r="O83" s="7" t="inlineStr"/>
+      <c r="P83" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10460,7 +10630,7 @@
           <t>3774975</t>
         </is>
       </c>
-      <c r="D84" s="24" t="n">
+      <c r="D84" s="28" t="n">
         <v>45855</v>
       </c>
       <c r="E84" s="7" t="inlineStr">
@@ -10485,7 +10655,7 @@
       <c r="J84" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K84" s="25" t="n">
+      <c r="K84" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L84" s="7" t="inlineStr">
@@ -10499,7 +10669,8 @@
         </is>
       </c>
       <c r="N84" s="7" t="inlineStr"/>
-      <c r="O84" s="7" t="inlineStr">
+      <c r="O84" s="7" t="inlineStr"/>
+      <c r="P84" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10521,7 +10692,7 @@
           <t>3774975</t>
         </is>
       </c>
-      <c r="D85" s="24" t="n">
+      <c r="D85" s="28" t="n">
         <v>45855</v>
       </c>
       <c r="E85" s="7" t="inlineStr">
@@ -10546,7 +10717,7 @@
       <c r="J85" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K85" s="25" t="n">
+      <c r="K85" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L85" s="7" t="inlineStr">
@@ -10560,7 +10731,8 @@
         </is>
       </c>
       <c r="N85" s="7" t="inlineStr"/>
-      <c r="O85" s="7" t="inlineStr">
+      <c r="O85" s="7" t="inlineStr"/>
+      <c r="P85" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10582,7 +10754,7 @@
           <t>3774976</t>
         </is>
       </c>
-      <c r="D86" s="24" t="n">
+      <c r="D86" s="28" t="n">
         <v>45866</v>
       </c>
       <c r="E86" s="7" t="inlineStr">
@@ -10607,7 +10779,7 @@
       <c r="J86" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K86" s="25" t="n">
+      <c r="K86" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L86" s="7" t="inlineStr">
@@ -10621,7 +10793,8 @@
         </is>
       </c>
       <c r="N86" s="7" t="inlineStr"/>
-      <c r="O86" s="7" t="inlineStr">
+      <c r="O86" s="7" t="inlineStr"/>
+      <c r="P86" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10643,7 +10816,7 @@
           <t>3774976</t>
         </is>
       </c>
-      <c r="D87" s="24" t="n">
+      <c r="D87" s="28" t="n">
         <v>45866</v>
       </c>
       <c r="E87" s="7" t="inlineStr">
@@ -10668,7 +10841,7 @@
       <c r="J87" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K87" s="25" t="n">
+      <c r="K87" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L87" s="7" t="inlineStr">
@@ -10682,7 +10855,8 @@
         </is>
       </c>
       <c r="N87" s="7" t="inlineStr"/>
-      <c r="O87" s="7" t="inlineStr">
+      <c r="O87" s="7" t="inlineStr"/>
+      <c r="P87" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10704,7 +10878,7 @@
           <t>3774976</t>
         </is>
       </c>
-      <c r="D88" s="24" t="n">
+      <c r="D88" s="28" t="n">
         <v>45866</v>
       </c>
       <c r="E88" s="7" t="inlineStr">
@@ -10729,7 +10903,7 @@
       <c r="J88" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K88" s="25" t="n">
+      <c r="K88" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L88" s="7" t="inlineStr">
@@ -10743,7 +10917,8 @@
         </is>
       </c>
       <c r="N88" s="7" t="inlineStr"/>
-      <c r="O88" s="7" t="inlineStr">
+      <c r="O88" s="7" t="inlineStr"/>
+      <c r="P88" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10765,7 +10940,7 @@
           <t>3774976</t>
         </is>
       </c>
-      <c r="D89" s="24" t="n">
+      <c r="D89" s="28" t="n">
         <v>45866</v>
       </c>
       <c r="E89" s="7" t="inlineStr">
@@ -10790,7 +10965,7 @@
       <c r="J89" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K89" s="25" t="n">
+      <c r="K89" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L89" s="7" t="inlineStr">
@@ -10804,7 +10979,8 @@
         </is>
       </c>
       <c r="N89" s="7" t="inlineStr"/>
-      <c r="O89" s="7" t="inlineStr">
+      <c r="O89" s="7" t="inlineStr"/>
+      <c r="P89" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10826,7 +11002,7 @@
           <t>3774976</t>
         </is>
       </c>
-      <c r="D90" s="24" t="n">
+      <c r="D90" s="28" t="n">
         <v>45866</v>
       </c>
       <c r="E90" s="7" t="inlineStr">
@@ -10851,7 +11027,7 @@
       <c r="J90" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K90" s="25" t="n">
+      <c r="K90" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L90" s="7" t="inlineStr">
@@ -10865,7 +11041,8 @@
         </is>
       </c>
       <c r="N90" s="7" t="inlineStr"/>
-      <c r="O90" s="7" t="inlineStr">
+      <c r="O90" s="7" t="inlineStr"/>
+      <c r="P90" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10887,7 +11064,7 @@
           <t>3774978</t>
         </is>
       </c>
-      <c r="D91" s="24" t="n">
+      <c r="D91" s="28" t="n">
         <v>45869</v>
       </c>
       <c r="E91" s="7" t="inlineStr">
@@ -10912,7 +11089,7 @@
       <c r="J91" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K91" s="25" t="n">
+      <c r="K91" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L91" s="7" t="inlineStr">
@@ -10922,7 +11099,8 @@
       </c>
       <c r="M91" s="7" t="inlineStr"/>
       <c r="N91" s="7" t="inlineStr"/>
-      <c r="O91" s="7" t="inlineStr">
+      <c r="O91" s="7" t="inlineStr"/>
+      <c r="P91" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -10944,7 +11122,7 @@
           <t>3774977</t>
         </is>
       </c>
-      <c r="D92" s="24" t="n">
+      <c r="D92" s="28" t="n">
         <v>45869</v>
       </c>
       <c r="E92" s="7" t="inlineStr">
@@ -10969,7 +11147,7 @@
       <c r="J92" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K92" s="25" t="n">
+      <c r="K92" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L92" s="7" t="inlineStr">
@@ -10983,7 +11161,8 @@
         </is>
       </c>
       <c r="N92" s="7" t="inlineStr"/>
-      <c r="O92" s="7" t="inlineStr">
+      <c r="O92" s="7" t="inlineStr"/>
+      <c r="P92" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -11005,7 +11184,7 @@
           <t>3774977</t>
         </is>
       </c>
-      <c r="D93" s="24" t="n">
+      <c r="D93" s="28" t="n">
         <v>45869</v>
       </c>
       <c r="E93" s="7" t="inlineStr">
@@ -11030,7 +11209,7 @@
       <c r="J93" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K93" s="25" t="n">
+      <c r="K93" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L93" s="7" t="inlineStr">
@@ -11044,7 +11223,8 @@
         </is>
       </c>
       <c r="N93" s="7" t="inlineStr"/>
-      <c r="O93" s="7" t="inlineStr">
+      <c r="O93" s="7" t="inlineStr"/>
+      <c r="P93" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -11066,7 +11246,7 @@
           <t>3774977</t>
         </is>
       </c>
-      <c r="D94" s="24" t="n">
+      <c r="D94" s="28" t="n">
         <v>45869</v>
       </c>
       <c r="E94" s="7" t="inlineStr">
@@ -11091,7 +11271,7 @@
       <c r="J94" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K94" s="25" t="n">
+      <c r="K94" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L94" s="7" t="inlineStr">
@@ -11105,7 +11285,8 @@
         </is>
       </c>
       <c r="N94" s="7" t="inlineStr"/>
-      <c r="O94" s="7" t="inlineStr">
+      <c r="O94" s="7" t="inlineStr"/>
+      <c r="P94" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -11127,7 +11308,7 @@
           <t>3774977</t>
         </is>
       </c>
-      <c r="D95" s="24" t="n">
+      <c r="D95" s="28" t="n">
         <v>45869</v>
       </c>
       <c r="E95" s="7" t="inlineStr">
@@ -11152,7 +11333,7 @@
       <c r="J95" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K95" s="25" t="n">
+      <c r="K95" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L95" s="7" t="inlineStr">
@@ -11166,7 +11347,8 @@
         </is>
       </c>
       <c r="N95" s="7" t="inlineStr"/>
-      <c r="O95" s="7" t="inlineStr">
+      <c r="O95" s="7" t="inlineStr"/>
+      <c r="P95" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -11188,7 +11370,7 @@
           <t>3776571</t>
         </is>
       </c>
-      <c r="D96" s="24" t="n">
+      <c r="D96" s="28" t="n">
         <v>45876</v>
       </c>
       <c r="E96" s="7" t="inlineStr">
@@ -11213,7 +11395,7 @@
       <c r="J96" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K96" s="25" t="n">
+      <c r="K96" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L96" s="7" t="inlineStr">
@@ -11227,7 +11409,8 @@
         </is>
       </c>
       <c r="N96" s="7" t="inlineStr"/>
-      <c r="O96" s="7" t="inlineStr">
+      <c r="O96" s="7" t="inlineStr"/>
+      <c r="P96" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -11249,7 +11432,7 @@
           <t>3776571</t>
         </is>
       </c>
-      <c r="D97" s="24" t="n">
+      <c r="D97" s="28" t="n">
         <v>45876</v>
       </c>
       <c r="E97" s="7" t="inlineStr">
@@ -11274,7 +11457,7 @@
       <c r="J97" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K97" s="25" t="n">
+      <c r="K97" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L97" s="7" t="inlineStr">
@@ -11288,7 +11471,8 @@
         </is>
       </c>
       <c r="N97" s="7" t="inlineStr"/>
-      <c r="O97" s="7" t="inlineStr">
+      <c r="O97" s="7" t="inlineStr"/>
+      <c r="P97" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -11310,7 +11494,7 @@
           <t>3776571</t>
         </is>
       </c>
-      <c r="D98" s="24" t="n">
+      <c r="D98" s="28" t="n">
         <v>45876</v>
       </c>
       <c r="E98" s="7" t="inlineStr">
@@ -11335,7 +11519,7 @@
       <c r="J98" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K98" s="25" t="n">
+      <c r="K98" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L98" s="7" t="inlineStr">
@@ -11349,7 +11533,8 @@
         </is>
       </c>
       <c r="N98" s="7" t="inlineStr"/>
-      <c r="O98" s="7" t="inlineStr">
+      <c r="O98" s="7" t="inlineStr"/>
+      <c r="P98" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -11371,7 +11556,7 @@
           <t>3776571</t>
         </is>
       </c>
-      <c r="D99" s="24" t="n">
+      <c r="D99" s="28" t="n">
         <v>45876</v>
       </c>
       <c r="E99" s="7" t="inlineStr">
@@ -11396,7 +11581,7 @@
       <c r="J99" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K99" s="25" t="n">
+      <c r="K99" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L99" s="7" t="inlineStr">
@@ -11410,7 +11595,8 @@
         </is>
       </c>
       <c r="N99" s="7" t="inlineStr"/>
-      <c r="O99" s="7" t="inlineStr">
+      <c r="O99" s="7" t="inlineStr"/>
+      <c r="P99" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -11432,7 +11618,7 @@
           <t>3776571</t>
         </is>
       </c>
-      <c r="D100" s="24" t="n">
+      <c r="D100" s="28" t="n">
         <v>45876</v>
       </c>
       <c r="E100" s="7" t="inlineStr">
@@ -11457,7 +11643,7 @@
       <c r="J100" s="10" t="n">
         <v>0</v>
       </c>
-      <c r="K100" s="25" t="n">
+      <c r="K100" s="29" t="n">
         <v>0</v>
       </c>
       <c r="L100" s="7" t="inlineStr">
@@ -11471,7 +11657,8 @@
         </is>
       </c>
       <c r="N100" s="7" t="inlineStr"/>
-      <c r="O100" s="7" t="inlineStr">
+      <c r="O100" s="7" t="inlineStr"/>
+      <c r="P100" s="7" t="inlineStr">
         <is>
           <t>±5%</t>
         </is>
@@ -11479,7 +11666,7 @@
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:O1"/>
+    <mergeCell ref="A1:P1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>